<commit_message>
criada a função de calcular a carga tributaria em porcentagem, alterado a escrita nas celulas da planilha
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,7 +449,377 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>ICMS CALCULADO</t>
+          <t>Carga Tributária (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>000043</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>14.500,00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000043.pdf</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:31.627339</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>11.16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>000044</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>21/05/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>15.800,00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000044.pdf</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:32.128959</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>000045</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>22/05/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>13.000,00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000045.pdf</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:32.793208</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>11.16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>000046</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>13.100,00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000046.pdf</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:33.278003</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>000047</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>29.500,00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000047.pdf</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:33.691483</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>000048</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>25/05/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>10.700,00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000048.pdf</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:34.091932</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>000049</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>26/05/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>13.800,00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000049.pdf</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:34.351681</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>11.16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>000050</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>27/05/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>18.200,00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000050.pdf</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:34.644306</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>11.15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>000051</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>23.300,00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nota_fiscal_000051.pdf</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:34.851041</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>11.16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>000042</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>19/05/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15.450,00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>nota_fiscal_exemplo.pdf</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-05-31 14:10:35.099497</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>11.15%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
totalizador dos valores das NF e escrita na celula
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,7 +481,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:31.627339</t>
+          <t>2026-05-31 14:38:48.602265</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:32.128959</t>
+          <t>2026-05-31 14:38:48.725791</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:32.793208</t>
+          <t>2026-05-31 14:38:48.888055</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:33.278003</t>
+          <t>2026-05-31 14:38:49.007526</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:33.691483</t>
+          <t>2026-05-31 14:38:49.117857</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:34.091932</t>
+          <t>2026-05-31 14:38:49.255168</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:34.351681</t>
+          <t>2026-05-31 14:38:49.395285</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:34.644306</t>
+          <t>2026-05-31 14:38:49.518471</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:34.851041</t>
+          <t>2026-05-31 14:38:49.632487</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -814,13 +814,23 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-31 14:10:35.099497</t>
+          <t>2026-05-31 14:38:49.769462</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>11.15%</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" t="n">
+        <v>151900</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="n">
+        <v>167350</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adicionado a verificação para ver se o arquivo xlsx existe, se sim, deletar e criar um novo
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:48.602265</t>
+          <t>2026-05-31 17:15:09.621561</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:48.725791</t>
+          <t>2026-05-31 17:15:09.793373</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:48.888055</t>
+          <t>2026-05-31 17:15:09.925663</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.007526</t>
+          <t>2026-05-31 17:15:10.067296</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.117857</t>
+          <t>2026-05-31 17:15:10.226292</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.255168</t>
+          <t>2026-05-31 17:15:10.408329</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.395285</t>
+          <t>2026-05-31 17:15:10.549524</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.518471</t>
+          <t>2026-05-31 17:15:10.699715</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.632487</t>
+          <t>2026-05-31 17:15:10.831127</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-31 14:38:49.769462</t>
+          <t>2026-05-31 17:15:11.013134</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
alteração no laço de repetição e no wb. save
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:09.621561</t>
+          <t>2026-06-01 15:22:58.019247</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:09.793373</t>
+          <t>2026-06-01 15:22:58.099398</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:09.925663</t>
+          <t>2026-06-01 15:22:58.193666</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.067296</t>
+          <t>2026-06-01 15:22:58.297773</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.226292</t>
+          <t>2026-06-01 15:22:58.399570</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.408329</t>
+          <t>2026-06-01 15:22:58.506271</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.549524</t>
+          <t>2026-06-01 15:22:58.617453</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.699715</t>
+          <t>2026-06-01 15:22:58.763389</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:10.831127</t>
+          <t>2026-06-01 15:22:58.903315</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -814,18 +814,13 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-05-31 17:15:11.013134</t>
+          <t>2026-06-01 15:22:59.006086</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>11.15%</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" t="n">
-        <v>151900</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
remover variavel nÕ UTILIZADA
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.019247</t>
+          <t>2026-06-01 15:25:16.890626</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.099398</t>
+          <t>2026-06-01 15:25:16.959785</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.193666</t>
+          <t>2026-06-01 15:25:17.048135</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.297773</t>
+          <t>2026-06-01 15:25:17.127782</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.399570</t>
+          <t>2026-06-01 15:25:17.199210</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.506271</t>
+          <t>2026-06-01 15:25:17.288374</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.617453</t>
+          <t>2026-06-01 15:25:17.356398</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.763389</t>
+          <t>2026-06-01 15:25:17.423067</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:58.903315</t>
+          <t>2026-06-01 15:25:17.489605</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22:59.006086</t>
+          <t>2026-06-01 15:25:17.576326</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
código ler_nf adaptado para funcionar no google colab
</commit_message>
<xml_diff>
--- a/dados_notas_fiscais.xlsx
+++ b/dados_notas_fiscais.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:16.890626</t>
+          <t>2026-06-01 16:51:58.451344</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:16.959785</t>
+          <t>2026-06-01 16:52:00.297591</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.048135</t>
+          <t>2026-06-01 16:52:01.612725</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.127782</t>
+          <t>2026-06-01 16:52:02.069685</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.199210</t>
+          <t>2026-06-01 16:52:02.428614</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.288374</t>
+          <t>2026-06-01 16:52:02.801214</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.356398</t>
+          <t>2026-06-01 16:52:03.113079</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.423067</t>
+          <t>2026-06-01 16:52:03.407352</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.489605</t>
+          <t>2026-06-01 16:52:03.713887</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-06-01 15:25:17.576326</t>
+          <t>2026-06-01 16:52:04.286113</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>